<commit_message>
Accept CMP Code header alias and add Fiber/FTTx format dropdown
Fiber uploads only read "MP Code" into the mp_code column, so a file
using "CMP Code" (CMP and MP are the same field, used interchangeably
across real files) silently lost that column. Also replaces the two
static format-download links in the upload modal with a single
Fiber/FTTx dropdown, and updates the fiber template to match the
current real-world header layout (single CIRCLE column, CMP/CMP Code).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/formats/fiber_format.xlsx
+++ b/frontend/public/formats/fiber_format.xlsx
@@ -397,25 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P3"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
-    <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="17.83203125" customWidth="1"/>
-    <col min="15" max="15" width="14.83203125" customWidth="1"/>
-    <col min="16" max="16" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:O3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -428,42 +410,39 @@
         <v>N/W</v>
       </c>
       <c r="D1" t="str">
-        <v>Circle</v>
+        <v>CIRCLE</v>
       </c>
       <c r="E1" t="str">
-        <v>CIRCLE</v>
+        <v>CMP</v>
       </c>
       <c r="F1" t="str">
-        <v>MP</v>
+        <v>CMP Code</v>
       </c>
       <c r="G1" t="str">
-        <v>MP Code</v>
+        <v>SPAN_TYPE</v>
       </c>
       <c r="H1" t="str">
-        <v>SPAN_TYPE</v>
+        <v>SPAN_LINK_ID</v>
       </c>
       <c r="I1" t="str">
-        <v>SPAN_LINK_ID</v>
+        <v>CMM Appd</v>
       </c>
       <c r="J1" t="str">
-        <v>CMM Appd</v>
+        <v>Status</v>
       </c>
       <c r="K1" t="str">
-        <v>Status</v>
+        <v>UG</v>
       </c>
       <c r="L1" t="str">
-        <v>UG</v>
+        <v>Aerial</v>
       </c>
       <c r="M1" t="str">
-        <v>Aerial</v>
+        <v>Patrolling Status</v>
       </c>
       <c r="N1" t="str">
-        <v>Patrolling Status</v>
+        <v>SP Name</v>
       </c>
       <c r="O1" t="str">
-        <v>SP Name</v>
-      </c>
-      <c r="P1" t="str">
         <v>Route Status</v>
       </c>
     </row>
@@ -481,39 +460,36 @@
         <v>Uttar Pradesh East</v>
       </c>
       <c r="E2" t="str">
-        <v>UE-2</v>
+        <v>6013</v>
       </c>
       <c r="F2" t="str">
-        <v>6013</v>
+        <v>INUEVRNS01</v>
       </c>
       <c r="G2" t="str">
-        <v>INUEVRNS01</v>
+        <v>INTRACITY</v>
       </c>
       <c r="H2" t="str">
-        <v>INTRACITY</v>
-      </c>
-      <c r="I2" t="str">
         <v>VRNS_6013</v>
       </c>
-      <c r="J2">
+      <c r="I2">
         <v>0</v>
       </c>
-      <c r="K2" t="str">
+      <c r="J2" t="str">
         <v>Approved</v>
       </c>
+      <c r="K2">
+        <v>0.12</v>
+      </c>
       <c r="L2">
-        <v>0.12</v>
-      </c>
-      <c r="M2">
         <v>0</v>
       </c>
+      <c r="M2" t="str">
+        <v>NA</v>
+      </c>
       <c r="N2" t="str">
-        <v>NA</v>
+        <v>SG Encon</v>
       </c>
       <c r="O2" t="str">
-        <v>SG Encon</v>
-      </c>
-      <c r="P2" t="str">
         <v>Live</v>
       </c>
     </row>
@@ -531,45 +507,42 @@
         <v>Delhi</v>
       </c>
       <c r="E3" t="str">
-        <v>DL</v>
+        <v>1042</v>
       </c>
       <c r="F3" t="str">
-        <v>1042</v>
+        <v>INDLROH02</v>
       </c>
       <c r="G3" t="str">
-        <v>INDLROH02</v>
+        <v>INTERCITY</v>
       </c>
       <c r="H3" t="str">
-        <v>INTERCITY</v>
-      </c>
-      <c r="I3" t="str">
         <v>DEL_1042</v>
       </c>
-      <c r="J3">
+      <c r="I3">
         <v>0</v>
       </c>
-      <c r="K3" t="str">
+      <c r="J3" t="str">
         <v>Approved</v>
       </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
       <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
         <v>3.4</v>
       </c>
+      <c r="M3" t="str">
+        <v>Done</v>
+      </c>
       <c r="N3" t="str">
-        <v>Done</v>
+        <v>SG Encon</v>
       </c>
       <c r="O3" t="str">
-        <v>SG Encon</v>
-      </c>
-      <c r="P3" t="str">
         <v>Live</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>